<commit_message>
Adding of 2 models and plotting all those together
</commit_message>
<xml_diff>
--- a/V3.xlsx
+++ b/V3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DE\sem 5\Codes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{980A9451-1284-414D-951D-DA9A5289152C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D8C6B8F-DC2D-4584-BBFB-D4EFFF7BE0D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-756" windowWidth="23256" windowHeight="12576" xr2:uid="{7DCB483B-EADE-468B-A11D-0B02376EF2F9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" xr2:uid="{7DCB483B-EADE-468B-A11D-0B02376EF2F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -7753,7 +7753,7 @@
       </c>
       <c r="C115" s="5">
         <f t="shared" si="2"/>
-        <v>92.314920000000001</v>
+        <v>92.315020000000004</v>
       </c>
       <c r="D115" s="2">
         <v>7.03</v>
@@ -7783,7 +7783,7 @@
         <v>6.8000000000000005E-4</v>
       </c>
       <c r="M115" s="2">
-        <v>5.9999999999999995E-4</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="N115" s="2">
         <v>0.128</v>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="C116" s="5">
         <f t="shared" si="2"/>
-        <v>92.314819999999997</v>
+        <v>92.315020000000004</v>
       </c>
       <c r="D116" s="2">
         <v>7.03</v>
@@ -7846,7 +7846,7 @@
         <v>6.8000000000000005E-4</v>
       </c>
       <c r="M116" s="2">
-        <v>6.9999999999999999E-4</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="N116" s="2">
         <v>0.128</v>
@@ -7879,7 +7879,7 @@
       </c>
       <c r="C117" s="5">
         <f t="shared" si="2"/>
-        <v>92.314719999999994</v>
+        <v>92.315020000000004</v>
       </c>
       <c r="D117" s="2">
         <v>7.03</v>
@@ -7909,7 +7909,7 @@
         <v>6.8000000000000005E-4</v>
       </c>
       <c r="M117" s="2">
-        <v>8.0000000000000004E-4</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="N117" s="2">
         <v>0.128</v>
@@ -7942,7 +7942,7 @@
       </c>
       <c r="C118" s="5">
         <f t="shared" si="2"/>
-        <v>92.314620000000005</v>
+        <v>92.315020000000004</v>
       </c>
       <c r="D118" s="2">
         <v>7.03</v>
@@ -7972,7 +7972,7 @@
         <v>6.8000000000000005E-4</v>
       </c>
       <c r="M118" s="2">
-        <v>8.9999999999999998E-4</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="N118" s="2">
         <v>0.128</v>
@@ -8005,7 +8005,7 @@
       </c>
       <c r="C119" s="5">
         <f t="shared" si="2"/>
-        <v>92.314520000000002</v>
+        <v>92.315020000000004</v>
       </c>
       <c r="D119" s="2">
         <v>7.03</v>
@@ -8035,7 +8035,7 @@
         <v>6.8000000000000005E-4</v>
       </c>
       <c r="M119" s="2">
-        <v>1E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="N119" s="2">
         <v>0.128</v>
@@ -8068,7 +8068,7 @@
       </c>
       <c r="C120" s="5">
         <f t="shared" si="2"/>
-        <v>92.314419999999998</v>
+        <v>92.315020000000004</v>
       </c>
       <c r="D120" s="2">
         <v>7.03</v>
@@ -8098,7 +8098,7 @@
         <v>6.8000000000000005E-4</v>
       </c>
       <c r="M120" s="2">
-        <v>1.1000000000000001E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="N120" s="2">
         <v>0.128</v>
@@ -8131,7 +8131,7 @@
       </c>
       <c r="C121" s="5">
         <f t="shared" si="2"/>
-        <v>92.314319999999995</v>
+        <v>92.315020000000004</v>
       </c>
       <c r="D121" s="2">
         <v>7.03</v>
@@ -8161,7 +8161,7 @@
         <v>6.8000000000000005E-4</v>
       </c>
       <c r="M121" s="2">
-        <v>1.1999999999999999E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="N121" s="2">
         <v>0.128</v>
@@ -8194,7 +8194,7 @@
       </c>
       <c r="C122" s="5">
         <f t="shared" si="2"/>
-        <v>92.314220000000006</v>
+        <v>92.315020000000004</v>
       </c>
       <c r="D122" s="2">
         <v>7.03</v>
@@ -8224,7 +8224,7 @@
         <v>6.8000000000000005E-4</v>
       </c>
       <c r="M122" s="2">
-        <v>1.2999999999999999E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="N122" s="2">
         <v>0.128</v>
@@ -8257,7 +8257,7 @@
       </c>
       <c r="C123" s="5">
         <f t="shared" si="2"/>
-        <v>92.314120000000003</v>
+        <v>92.315020000000004</v>
       </c>
       <c r="D123" s="2">
         <v>7.03</v>
@@ -8287,7 +8287,7 @@
         <v>6.8000000000000005E-4</v>
       </c>
       <c r="M123" s="2">
-        <v>1.4E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="N123" s="2">
         <v>0.128</v>
@@ -8320,7 +8320,7 @@
       </c>
       <c r="C124" s="5">
         <f t="shared" si="2"/>
-        <v>92.314019999999999</v>
+        <v>92.315020000000004</v>
       </c>
       <c r="D124" s="2">
         <v>7.03</v>
@@ -8350,7 +8350,7 @@
         <v>6.8000000000000005E-4</v>
       </c>
       <c r="M124" s="2">
-        <v>1.5E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="N124" s="2">
         <v>0.128</v>
@@ -8383,7 +8383,7 @@
       </c>
       <c r="C125" s="5">
         <f t="shared" si="2"/>
-        <v>92.313919999999996</v>
+        <v>92.315020000000004</v>
       </c>
       <c r="D125" s="2">
         <v>7.03</v>
@@ -8413,7 +8413,7 @@
         <v>6.8000000000000005E-4</v>
       </c>
       <c r="M125" s="2">
-        <v>1.6000000000000001E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="N125" s="2">
         <v>0.128</v>
@@ -8446,7 +8446,7 @@
       </c>
       <c r="C126" s="5">
         <f t="shared" si="2"/>
-        <v>92.313820000000007</v>
+        <v>92.315020000000004</v>
       </c>
       <c r="D126" s="2">
         <v>7.03</v>
@@ -8476,7 +8476,7 @@
         <v>6.8000000000000005E-4</v>
       </c>
       <c r="M126" s="2">
-        <v>1.6999999999999999E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="N126" s="2">
         <v>0.128</v>
@@ -8509,7 +8509,7 @@
       </c>
       <c r="C127" s="5">
         <f t="shared" si="2"/>
-        <v>92.313720000000004</v>
+        <v>92.315020000000004</v>
       </c>
       <c r="D127" s="2">
         <v>7.03</v>
@@ -8539,7 +8539,7 @@
         <v>6.8000000000000005E-4</v>
       </c>
       <c r="M127" s="2">
-        <v>1.8E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="N127" s="2">
         <v>0.128</v>
@@ -8572,7 +8572,7 @@
       </c>
       <c r="C128" s="5">
         <f t="shared" si="2"/>
-        <v>92.31362</v>
+        <v>92.315020000000004</v>
       </c>
       <c r="D128" s="2">
         <v>7.03</v>
@@ -8602,7 +8602,7 @@
         <v>6.8000000000000005E-4</v>
       </c>
       <c r="M128" s="2">
-        <v>1.9E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="N128" s="2">
         <v>0.128</v>
@@ -8635,7 +8635,7 @@
       </c>
       <c r="C129" s="5">
         <f t="shared" si="2"/>
-        <v>92.313519999999997</v>
+        <v>92.315020000000004</v>
       </c>
       <c r="D129" s="2">
         <v>7.03</v>
@@ -8665,7 +8665,7 @@
         <v>6.8000000000000005E-4</v>
       </c>
       <c r="M129" s="2">
-        <v>2E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="N129" s="2">
         <v>0.128</v>
@@ -8698,7 +8698,7 @@
       </c>
       <c r="C130" s="5">
         <f t="shared" si="2"/>
-        <v>92.313419999999994</v>
+        <v>92.315020000000004</v>
       </c>
       <c r="D130" s="2">
         <v>7.03</v>
@@ -8728,7 +8728,7 @@
         <v>6.8000000000000005E-4</v>
       </c>
       <c r="M130" s="2">
-        <v>2.0999999999999999E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="N130" s="2">
         <v>0.128</v>
@@ -8761,7 +8761,7 @@
       </c>
       <c r="C131" s="5">
         <f t="shared" si="2"/>
-        <v>92.313320000000004</v>
+        <v>92.315020000000004</v>
       </c>
       <c r="D131" s="2">
         <v>7.03</v>
@@ -8791,7 +8791,7 @@
         <v>6.8000000000000005E-4</v>
       </c>
       <c r="M131" s="2">
-        <v>2.2000000000000001E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="N131" s="2">
         <v>0.128</v>
@@ -8824,7 +8824,7 @@
       </c>
       <c r="C132" s="5">
         <f t="shared" ref="C132:C169" si="3">100-SUM(D132:N132)</f>
-        <v>92.313220000000001</v>
+        <v>92.315020000000004</v>
       </c>
       <c r="D132" s="2">
         <v>7.03</v>
@@ -8854,7 +8854,7 @@
         <v>6.8000000000000005E-4</v>
       </c>
       <c r="M132" s="2">
-        <v>2.3E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="N132" s="2">
         <v>0.128</v>
@@ -8887,7 +8887,7 @@
       </c>
       <c r="C133" s="5">
         <f t="shared" si="3"/>
-        <v>92.313119999999998</v>
+        <v>92.315020000000004</v>
       </c>
       <c r="D133" s="2">
         <v>7.03</v>
@@ -8917,7 +8917,7 @@
         <v>6.8000000000000005E-4</v>
       </c>
       <c r="M133" s="2">
-        <v>2.3999999999999998E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="N133" s="2">
         <v>0.128</v>
@@ -8950,7 +8950,7 @@
       </c>
       <c r="C134" s="5">
         <f t="shared" si="3"/>
-        <v>92.313019999999995</v>
+        <v>92.315020000000004</v>
       </c>
       <c r="D134" s="2">
         <v>7.03</v>
@@ -8980,7 +8980,7 @@
         <v>6.8000000000000005E-4</v>
       </c>
       <c r="M134" s="2">
-        <v>2.5000000000000001E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="N134" s="2">
         <v>0.128</v>

</xml_diff>